<commit_message>
reto 10 completado, consultar productos desde postman
</commit_message>
<xml_diff>
--- a/rws respaldo excel.xlsx
+++ b/rws respaldo excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\cositas\krake\INVENTARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E77CC260-3CEE-45E7-8D5A-A68C8B758F71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E43B6E5A-73F5-4744-8E83-BF7C90F2F1FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0DB715EB-206E-4D13-9055-4FF6D40D2BDF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
   <si>
     <t>accion</t>
   </si>
@@ -60,6 +60,24 @@
   </si>
   <si>
     <t xml:space="preserve">Recupera todos los tipos de documentos </t>
+  </si>
+  <si>
+    <t>POST</t>
+  </si>
+  <si>
+    <t>/proveedores/crear</t>
+  </si>
+  <si>
+    <t>Crea un proovedor</t>
+  </si>
+  <si>
+    <t>GET</t>
+  </si>
+  <si>
+    <t>recupera todos los productos cuyo nombre contenga la subcadena</t>
+  </si>
+  <si>
+    <t>/productos/buscar/{subcadena}</t>
   </si>
 </sst>
 </file>
@@ -431,7 +449,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E244D5B-8611-4749-A511-7C8896414761}">
-  <dimension ref="B2:D4"/>
+  <dimension ref="B2:D6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="7" bestFit="1" customWidth="1"/>
@@ -472,6 +490,28 @@
         <v>7</v>
       </c>
     </row>
+    <row r="5" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" t="s">
+        <v>12</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
correccion de los set ya que enviaba otra info, y completo el reto 11
</commit_message>
<xml_diff>
--- a/rws respaldo excel.xlsx
+++ b/rws respaldo excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\cositas\krake\INVENTARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E43B6E5A-73F5-4744-8E83-BF7C90F2F1FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9D07BCA-7845-445C-AF29-97DC1E638E70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0DB715EB-206E-4D13-9055-4FF6D40D2BDF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
   <si>
     <t>accion</t>
   </si>
@@ -78,6 +78,12 @@
   </si>
   <si>
     <t>/productos/buscar/{subcadena}</t>
+  </si>
+  <si>
+    <t>/productos/crear</t>
+  </si>
+  <si>
+    <t>Crea un producto</t>
   </si>
 </sst>
 </file>
@@ -449,7 +455,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E244D5B-8611-4749-A511-7C8896414761}">
-  <dimension ref="B2:D6"/>
+  <dimension ref="B2:D7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="7" bestFit="1" customWidth="1"/>
@@ -512,6 +518,17 @@
         <v>12</v>
       </c>
     </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>